<commit_message>
Calcuating Dwell Times for Organs
</commit_message>
<xml_diff>
--- a/FlowTracker.xlsx
+++ b/FlowTracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbnor\Documents\Full Body Flow Model Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\PHSAhome2.phsabc.ehcnet.ca\Cassidy.Northway\Remote Git\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28FA70EC-6427-4046-8F80-A1BDD186CBB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE0B03A2-17C1-49EB-B3DA-3FF6E79BC826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21697" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-4770" windowWidth="18240" windowHeight="28440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="arteries" sheetId="1" r:id="rId1"/>
@@ -18,18 +18,30 @@
     <sheet name="veins-inf" sheetId="5" r:id="rId3"/>
     <sheet name="PulArt" sheetId="4" r:id="rId4"/>
     <sheet name="A-V Mapping" sheetId="6" r:id="rId5"/>
+    <sheet name="Dwell Time Calcs" sheetId="7" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2398" uniqueCount="862">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2410" uniqueCount="867">
   <si>
     <t>Filename</t>
   </si>
@@ -2500,9 +2512,6 @@
     <t>Brain</t>
   </si>
   <si>
-    <t xml:space="preserve">2015_Mynard SuppMaterial </t>
-  </si>
-  <si>
     <t>Stomach</t>
   </si>
   <si>
@@ -2587,41 +2596,59 @@
     <t>L Intenstine</t>
   </si>
   <si>
-    <t>1996_Legget Dwell Time Organs</t>
-  </si>
-  <si>
-    <t>Total Blood Volume (ml) 1996_legget</t>
-  </si>
-  <si>
-    <t>5300 mL</t>
-  </si>
-  <si>
-    <t>Caridac Output (mL/min) 1996_Legget</t>
-  </si>
-  <si>
-    <t>6500 ml/min</t>
-  </si>
-  <si>
-    <t>% Total BV</t>
-  </si>
-  <si>
-    <t>% CO Recived</t>
-  </si>
-  <si>
-    <t>3.8, 0.6</t>
-  </si>
-  <si>
-    <t>10, 1</t>
-  </si>
-  <si>
-    <t>25.5 (total)</t>
+    <t>Organ</t>
+  </si>
+  <si>
+    <t>S Intestines</t>
+  </si>
+  <si>
+    <t>Pancreas</t>
+  </si>
+  <si>
+    <t>L Intestines</t>
+  </si>
+  <si>
+    <t>Liver (From organs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liver </t>
+  </si>
+  <si>
+    <t>% Total Blood Volume</t>
+  </si>
+  <si>
+    <t>%  of Cardiac Output</t>
+  </si>
+  <si>
+    <t>Total BV (mL)</t>
+  </si>
+  <si>
+    <t>Cardiac Output (mL/min)</t>
+  </si>
+  <si>
+    <t>1996_legget</t>
+  </si>
+  <si>
+    <t>Dwell Time (A&gt;O&gt;V) (min)</t>
+  </si>
+  <si>
+    <t>Dwell Time (s)</t>
+  </si>
+  <si>
+    <t>ICRP 89</t>
+  </si>
+  <si>
+    <t>2010_Eipel</t>
+  </si>
+  <si>
+    <t>Name</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2635,8 +2662,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2645,19 +2678,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2686,12 +2725,12 @@
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2739,9 +2778,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2779,7 +2818,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2885,7 +2924,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3027,7 +3066,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -6101,7 +6140,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="I10" t="s">
         <v>11</v>
@@ -6125,7 +6164,7 @@
         <v>791</v>
       </c>
       <c r="D13" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
   </sheetData>
@@ -11249,562 +11288,1123 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{188388E5-F9D8-4148-BF34-9C51095EB628}">
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:U44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="3" max="3" width="23.140625" customWidth="1"/>
-    <col min="4" max="4" width="24.5703125" customWidth="1"/>
-    <col min="5" max="5" width="36.7109375" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" customWidth="1"/>
-    <col min="7" max="8" width="9.140625" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="27" customWidth="1"/>
+    <col min="1" max="1" width="28.28515625" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" customWidth="1"/>
+    <col min="5" max="5" width="24.5703125" customWidth="1"/>
+    <col min="6" max="6" width="36.7109375" customWidth="1"/>
+    <col min="7" max="7" width="26.5703125" customWidth="1"/>
+    <col min="8" max="9" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>866</v>
+      </c>
+      <c r="B1" t="s">
         <v>802</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>803</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>820</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="E1" s="4" t="s">
         <v>821</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>857</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>858</v>
-      </c>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="2" t="s">
-        <v>853</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>804</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>822</v>
+      </c>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>805</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>822</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>806</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>807</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>822</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>806</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>806</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>18</v>
+      </c>
+      <c r="D8" t="s">
+        <v>808</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>849</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B9">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>811</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>823</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>804</v>
-      </c>
-      <c r="D2" s="7" t="s">
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="2"/>
+      <c r="T9" s="2"/>
+      <c r="U9" s="2"/>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>21</v>
+      </c>
+      <c r="D10" t="s">
+        <v>809</v>
+      </c>
+      <c r="E10" s="4"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="2"/>
+      <c r="T10" s="2"/>
+      <c r="U10" s="2"/>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>24</v>
+      </c>
+      <c r="D11" t="s">
+        <v>810</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>810</v>
+      </c>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
+        <v>812</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>824</v>
+      </c>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="2"/>
+      <c r="T12" s="2"/>
+      <c r="U12" s="2"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B13">
+        <v>26</v>
+      </c>
+      <c r="D13" t="s">
+        <v>813</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>825</v>
+      </c>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+      <c r="S13" s="2"/>
+      <c r="T13" s="2"/>
+      <c r="U13" s="2"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B14">
+        <v>27</v>
+      </c>
+      <c r="D14" t="s">
+        <v>809</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="2"/>
+      <c r="T14" s="2"/>
+      <c r="U14" s="2"/>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B15">
+        <v>28</v>
+      </c>
+      <c r="D15" t="s">
+        <v>809</v>
+      </c>
+      <c r="E15" s="4"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="2"/>
+      <c r="T15" s="2"/>
+      <c r="U15" s="2"/>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B16">
+        <v>30</v>
+      </c>
+      <c r="D16" t="s">
+        <v>814</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>814</v>
+      </c>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2"/>
+      <c r="S16" s="2"/>
+      <c r="T16" s="2"/>
+      <c r="U16" s="2"/>
+    </row>
+    <row r="17" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <v>32</v>
+      </c>
+      <c r="D17" t="s">
+        <v>815</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>850</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="2"/>
+      <c r="T17" s="2"/>
+      <c r="U17" s="2"/>
+    </row>
+    <row r="18" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>35</v>
+      </c>
+      <c r="D18" t="s">
+        <v>816</v>
+      </c>
+      <c r="E18" s="4"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
+      <c r="U18" s="2"/>
+    </row>
+    <row r="19" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>37</v>
+      </c>
+      <c r="D19" t="s">
+        <v>817</v>
+      </c>
+      <c r="E19" s="4"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="2"/>
+      <c r="T19" s="2"/>
+      <c r="U19" s="2"/>
+    </row>
+    <row r="20" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>40</v>
+      </c>
+      <c r="D20" t="s">
+        <v>818</v>
+      </c>
+      <c r="E20" s="4"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="2"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2"/>
+      <c r="S20" s="2"/>
+      <c r="T20" s="2"/>
+      <c r="U20" s="2"/>
+    </row>
+    <row r="21" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B21">
+        <v>42</v>
+      </c>
+      <c r="D21" t="s">
+        <v>819</v>
+      </c>
+      <c r="E21" s="4"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2"/>
+      <c r="S21" s="2"/>
+      <c r="T21" s="2"/>
+      <c r="U21" s="2"/>
+    </row>
+    <row r="22" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <v>43</v>
+      </c>
+      <c r="D22" t="s">
+        <v>818</v>
+      </c>
+      <c r="E22" s="4"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
+      <c r="P22" s="2"/>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="2"/>
+      <c r="S22" s="2"/>
+      <c r="T22" s="2"/>
+      <c r="U22" s="2"/>
+    </row>
+    <row r="23" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B23">
+        <v>44</v>
+      </c>
+      <c r="D23" t="s">
+        <v>818</v>
+      </c>
+      <c r="E23" s="4"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
+      <c r="O23" s="2"/>
+      <c r="P23" s="2"/>
+      <c r="Q23" s="2"/>
+      <c r="R23" s="2"/>
+      <c r="S23" s="2"/>
+      <c r="T23" s="2"/>
+      <c r="U23" s="2"/>
+    </row>
+    <row r="24" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <v>45</v>
+      </c>
+      <c r="D24" t="s">
+        <v>819</v>
+      </c>
+      <c r="E24" s="4"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
+      <c r="O24" s="2"/>
+      <c r="P24" s="2"/>
+      <c r="Q24" s="2"/>
+      <c r="R24" s="2"/>
+      <c r="S24" s="2"/>
+      <c r="T24" s="2"/>
+      <c r="U24" s="2"/>
+    </row>
+    <row r="25" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B25">
+        <v>46</v>
+      </c>
+      <c r="D25" t="s">
+        <v>819</v>
+      </c>
+      <c r="E25" s="4"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
+      <c r="O25" s="2"/>
+      <c r="P25" s="2"/>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2"/>
+      <c r="S25" s="2"/>
+      <c r="T25" s="2"/>
+      <c r="U25" s="2"/>
+    </row>
+    <row r="26" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>826</v>
+      </c>
+      <c r="D26" t="s">
+        <v>834</v>
+      </c>
+      <c r="E26" t="s">
         <v>822</v>
       </c>
-      <c r="E2" s="5">
-        <v>1.2</v>
-      </c>
-      <c r="F2" s="5">
-        <v>12</v>
-      </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="2" t="s">
-        <v>854</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>805</v>
-      </c>
-      <c r="D3" s="7" t="s">
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
+      <c r="O26" s="2"/>
+      <c r="P26" s="2"/>
+      <c r="Q26" s="2"/>
+      <c r="R26" s="2"/>
+      <c r="S26" s="2"/>
+      <c r="T26" s="2"/>
+      <c r="U26" s="2"/>
+    </row>
+    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>827</v>
+      </c>
+      <c r="D27" t="s">
+        <v>835</v>
+      </c>
+      <c r="E27" t="s">
         <v>822</v>
       </c>
-      <c r="E3" s="5">
-        <v>1.2</v>
-      </c>
-      <c r="F3" s="5">
-        <v>12</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="3" t="s">
-        <v>855</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>852</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>828</v>
+      </c>
+      <c r="D28" t="s">
         <v>806</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="3" t="s">
-        <v>856</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>807</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>822</v>
-      </c>
-      <c r="E5" s="6">
-        <v>1.2</v>
-      </c>
-      <c r="F5" s="6">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
+    </row>
+    <row r="29" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>829</v>
+      </c>
+      <c r="D29" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="30" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>830</v>
+      </c>
+      <c r="D30" t="s">
         <v>806</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s">
+    </row>
+    <row r="31" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
+        <v>831</v>
+      </c>
+      <c r="D31" t="s">
         <v>806</v>
       </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
-        <v>808</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>850</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>859</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>860</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>811</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>824</v>
-      </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>21</v>
-      </c>
-      <c r="C10" t="s">
+    </row>
+    <row r="32" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
+        <v>832</v>
+      </c>
+      <c r="D32" t="s">
         <v>809</v>
       </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>24</v>
-      </c>
-      <c r="C11" t="s">
-        <v>810</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>810</v>
-      </c>
-      <c r="E11" s="6">
-        <v>2</v>
-      </c>
-      <c r="F11" s="6">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>25</v>
-      </c>
-      <c r="C12" t="s">
-        <v>812</v>
-      </c>
-      <c r="D12" s="7" t="s">
+    </row>
+    <row r="33" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
+        <v>833</v>
+      </c>
+      <c r="D33" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="34" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C34" t="s">
+        <v>836</v>
+      </c>
+      <c r="D34" t="s">
         <v>825</v>
       </c>
-      <c r="E12" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="F12" s="6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>26</v>
-      </c>
-      <c r="C13" t="s">
-        <v>813</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>826</v>
-      </c>
-      <c r="E13" s="6">
-        <v>10</v>
-      </c>
-      <c r="F13" s="6">
-        <v>6.5</v>
-      </c>
-      <c r="I13" t="s">
-        <v>861</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>27</v>
-      </c>
-      <c r="C14" t="s">
-        <v>809</v>
-      </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>28</v>
-      </c>
-      <c r="C15" t="s">
-        <v>809</v>
-      </c>
-      <c r="D15" s="7"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>30</v>
-      </c>
-      <c r="C16" t="s">
-        <v>814</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>814</v>
-      </c>
-      <c r="E16" s="5">
-        <v>2</v>
-      </c>
-      <c r="F16" s="5">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>32</v>
-      </c>
-      <c r="C17" t="s">
-        <v>815</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>851</v>
-      </c>
-      <c r="E17" s="5">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="F17" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>35</v>
-      </c>
-      <c r="C18" t="s">
-        <v>816</v>
-      </c>
-      <c r="D18" s="7"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>37</v>
-      </c>
-      <c r="C19" t="s">
-        <v>817</v>
-      </c>
-      <c r="D19" s="7"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>40</v>
-      </c>
-      <c r="C20" t="s">
-        <v>818</v>
-      </c>
-      <c r="D20" s="7"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>42</v>
-      </c>
-      <c r="C21" t="s">
-        <v>819</v>
-      </c>
-      <c r="D21" s="7"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>43</v>
-      </c>
-      <c r="C22" t="s">
-        <v>818</v>
-      </c>
-      <c r="D22" s="7"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>44</v>
-      </c>
-      <c r="C23" t="s">
-        <v>818</v>
-      </c>
-      <c r="D23" s="7"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>45</v>
-      </c>
-      <c r="C24" t="s">
-        <v>819</v>
-      </c>
-      <c r="D24" s="7"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>46</v>
-      </c>
-      <c r="C25" t="s">
-        <v>819</v>
-      </c>
-      <c r="D25" s="7"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>827</v>
-      </c>
-      <c r="C26" t="s">
-        <v>835</v>
-      </c>
-      <c r="D26" t="s">
-        <v>822</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>828</v>
-      </c>
-      <c r="C27" t="s">
-        <v>836</v>
-      </c>
-      <c r="D27" t="s">
-        <v>822</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
-        <v>829</v>
-      </c>
-      <c r="C28" t="s">
-        <v>806</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
-        <v>830</v>
-      </c>
-      <c r="C29" t="s">
-        <v>809</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
-        <v>831</v>
-      </c>
-      <c r="C30" t="s">
-        <v>806</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>832</v>
-      </c>
-      <c r="C31" t="s">
-        <v>806</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>833</v>
-      </c>
-      <c r="C32" t="s">
-        <v>809</v>
-      </c>
-    </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
-        <v>834</v>
-      </c>
-      <c r="C33" t="s">
-        <v>809</v>
-      </c>
-    </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B34" t="s">
+      <c r="E34" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="35" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C35" t="s">
         <v>837</v>
       </c>
-      <c r="C34" t="s">
-        <v>826</v>
-      </c>
-      <c r="D34" t="s">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
+      <c r="D35" t="s">
+        <v>825</v>
+      </c>
+      <c r="E35" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="36" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C36" t="s">
         <v>838</v>
       </c>
-      <c r="C35" t="s">
-        <v>826</v>
-      </c>
-      <c r="D35" t="s">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
+      <c r="D36" t="s">
+        <v>825</v>
+      </c>
+      <c r="E36" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="37" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C37" t="s">
         <v>839</v>
-      </c>
-      <c r="C36" t="s">
-        <v>826</v>
-      </c>
-      <c r="D36" t="s">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B37" t="s">
-        <v>840</v>
-      </c>
-      <c r="C37" t="s">
-        <v>814</v>
       </c>
       <c r="D37" t="s">
         <v>814</v>
       </c>
-    </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B38" t="s">
-        <v>841</v>
-      </c>
+      <c r="E37" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="38" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
-        <v>810</v>
+        <v>840</v>
       </c>
       <c r="D38" t="s">
         <v>810</v>
       </c>
-    </row>
-    <row r="39" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B39" t="s">
+      <c r="E38" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="39" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>846</v>
+      </c>
+      <c r="D39" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="40" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C40" t="s">
+        <v>841</v>
+      </c>
+      <c r="D40" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="41" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
+        <v>842</v>
+      </c>
+      <c r="D41" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="42" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C42" t="s">
+        <v>843</v>
+      </c>
+      <c r="D42" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="43" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C43" t="s">
         <v>847</v>
       </c>
-      <c r="C39" t="s">
-        <v>816</v>
-      </c>
-    </row>
-    <row r="40" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B40" t="s">
-        <v>842</v>
-      </c>
-      <c r="C40" t="s">
-        <v>817</v>
-      </c>
-    </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B41" t="s">
-        <v>843</v>
-      </c>
-      <c r="C41" t="s">
-        <v>818</v>
-      </c>
-    </row>
-    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B42" t="s">
-        <v>844</v>
-      </c>
-      <c r="C42" t="s">
-        <v>818</v>
-      </c>
-    </row>
-    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B43" t="s">
+      <c r="D43" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="44" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C44" t="s">
         <v>848</v>
       </c>
-      <c r="C43" t="s">
-        <v>819</v>
-      </c>
-    </row>
-    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B44" t="s">
-        <v>849</v>
-      </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>819</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F665A280-B941-4509-8B0A-1E2E1E43C816}">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="39.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" customWidth="1"/>
+    <col min="4" max="4" width="30.140625" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+    <col min="7" max="7" width="23.85546875" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>851</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>857</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>858</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>862</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>863</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>859</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>860</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>822</v>
+      </c>
+      <c r="B2">
+        <v>1.2</v>
+      </c>
+      <c r="C2">
+        <v>12</v>
+      </c>
+      <c r="D2">
+        <f>($F$2*B2)/($G$2*C2)</f>
+        <v>8.1538461538461532E-2</v>
+      </c>
+      <c r="E2" s="7">
+        <f>D2*60</f>
+        <v>4.8923076923076918</v>
+      </c>
+      <c r="F2">
+        <v>5300</v>
+      </c>
+      <c r="G2">
+        <v>6500</v>
+      </c>
+      <c r="I2" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>852</v>
+      </c>
+      <c r="B3">
+        <v>3.8</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <f t="shared" ref="D3:D11" si="0">($F$2*B3)/($G$2*C3)</f>
+        <v>0.30984615384615383</v>
+      </c>
+      <c r="E3" s="7">
+        <f>D3*60 +E11</f>
+        <v>37.902510121457489</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>853</v>
+      </c>
+      <c r="B4">
+        <v>0.6</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>0.48923076923076925</v>
+      </c>
+      <c r="E4" s="7">
+        <f>D4*60</f>
+        <v>29.353846153846156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>823</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>0.81538461538461537</v>
+      </c>
+      <c r="E5" s="7">
+        <f>D5*60 +E11</f>
+        <v>68.234817813765176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>810</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>19</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>8.5829959514170037E-2</v>
+      </c>
+      <c r="E6" s="7">
+        <f t="shared" ref="E3:E11" si="1">D6*60</f>
+        <v>5.1497975708502022</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>824</v>
+      </c>
+      <c r="B7">
+        <v>1.4</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>0.38051282051282048</v>
+      </c>
+      <c r="E7" s="7">
+        <f>D7*60+E11</f>
+        <v>42.142510121457491</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>854</v>
+      </c>
+      <c r="B8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>0.44846153846153852</v>
+      </c>
+      <c r="E8" s="7">
+        <f>D8*60 + E11</f>
+        <v>46.219433198380571</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>814</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>19</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>8.5829959514170037E-2</v>
+      </c>
+      <c r="E9" s="7">
+        <f t="shared" si="1"/>
+        <v>5.1497975708502022</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>856</v>
+      </c>
+      <c r="B10">
+        <f>10/4</f>
+        <v>2.5</v>
+      </c>
+      <c r="C10">
+        <v>6.5</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>0.31360946745562129</v>
+      </c>
+      <c r="E10" s="7">
+        <f t="shared" si="1"/>
+        <v>18.816568047337277</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>855</v>
+      </c>
+      <c r="B11">
+        <f>3*10/4</f>
+        <v>7.5</v>
+      </c>
+      <c r="C11">
+        <f>25.5-6.5</f>
+        <v>19</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>0.32186234817813764</v>
+      </c>
+      <c r="E11" s="7">
+        <f t="shared" si="1"/>
+        <v>19.311740890688259</v>
+      </c>
+      <c r="I11" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Prepping Data for BV Simulation
</commit_message>
<xml_diff>
--- a/FlowTracker.xlsx
+++ b/FlowTracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbnor\Documents\Full Body Flow Model Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46257476-5D13-4CE3-A2A4-04C9D95340FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF2329E-AAE3-4721-8746-92FC78FBE3CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3186,9 +3186,6 @@
     <t>2;82;85;0;4.89</t>
   </si>
   <si>
-    <t>0;126;126;0;1</t>
-  </si>
-  <si>
     <t>1;28;28;0;1</t>
   </si>
   <si>
@@ -3562,6 +3559,9 @@
   </si>
   <si>
     <t>126;98;99;0;0</t>
+  </si>
+  <si>
+    <t>0;126;126;0;0.955</t>
   </si>
 </sst>
 </file>
@@ -4013,7 +4013,7 @@
         <v>936</v>
       </c>
       <c r="B2" t="s">
-        <v>1047</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
@@ -4021,7 +4021,7 @@
         <v>935</v>
       </c>
       <c r="B3" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
@@ -4037,7 +4037,7 @@
         <v>844</v>
       </c>
       <c r="B5" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
@@ -4045,7 +4045,7 @@
         <v>845</v>
       </c>
       <c r="B6" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
@@ -4053,7 +4053,7 @@
         <v>818</v>
       </c>
       <c r="B7" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
@@ -4061,7 +4061,7 @@
         <v>807</v>
       </c>
       <c r="B8" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
@@ -4069,7 +4069,7 @@
         <v>819</v>
       </c>
       <c r="B9" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
@@ -4077,7 +4077,7 @@
         <v>846</v>
       </c>
       <c r="B10" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
@@ -4085,7 +4085,7 @@
         <v>811</v>
       </c>
       <c r="B11" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
@@ -4093,7 +4093,7 @@
         <v>848</v>
       </c>
       <c r="B12" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
@@ -4101,7 +4101,7 @@
         <v>847</v>
       </c>
       <c r="B13" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
@@ -4109,7 +4109,7 @@
         <v>1007</v>
       </c>
       <c r="B14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
@@ -4117,7 +4117,7 @@
         <v>1008</v>
       </c>
       <c r="B15" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.45">
@@ -4125,7 +4125,7 @@
         <v>1009</v>
       </c>
       <c r="B16" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.45">
@@ -4133,7 +4133,7 @@
         <v>1010</v>
       </c>
       <c r="B17" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.45">
@@ -4141,7 +4141,7 @@
         <v>1022</v>
       </c>
       <c r="B18" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.45">
@@ -4149,7 +4149,7 @@
         <v>1011</v>
       </c>
       <c r="B19" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.45">
@@ -4157,7 +4157,7 @@
         <v>1014</v>
       </c>
       <c r="B20" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.45">
@@ -4165,7 +4165,7 @@
         <v>1015</v>
       </c>
       <c r="B21" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.45">
@@ -4173,7 +4173,7 @@
         <v>1016</v>
       </c>
       <c r="B22" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.45">
@@ -4181,7 +4181,7 @@
         <v>1017</v>
       </c>
       <c r="B23" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.45">
@@ -4189,7 +4189,7 @@
         <v>1018</v>
       </c>
       <c r="B24" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.45">
@@ -4197,7 +4197,7 @@
         <v>1019</v>
       </c>
       <c r="B25" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.45">
@@ -4205,7 +4205,7 @@
         <v>1020</v>
       </c>
       <c r="B26" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.45">
@@ -4213,7 +4213,7 @@
         <v>1021</v>
       </c>
       <c r="B27" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.45">
@@ -4221,7 +4221,7 @@
         <v>1012</v>
       </c>
       <c r="B28" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.45">
@@ -4229,7 +4229,7 @@
         <v>1013</v>
       </c>
       <c r="B29" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.45">
@@ -4237,7 +4237,7 @@
         <v>963</v>
       </c>
       <c r="B30" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.45">
@@ -4245,7 +4245,7 @@
         <v>964</v>
       </c>
       <c r="B31" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.45">
@@ -4253,7 +4253,7 @@
         <v>965</v>
       </c>
       <c r="B32" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.45">
@@ -4261,7 +4261,7 @@
         <v>966</v>
       </c>
       <c r="B33" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.45">
@@ -4269,7 +4269,7 @@
         <v>967</v>
       </c>
       <c r="B34" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.45">
@@ -4277,7 +4277,7 @@
         <v>968</v>
       </c>
       <c r="B35" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.45">
@@ -4285,7 +4285,7 @@
         <v>969</v>
       </c>
       <c r="B36" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.45">
@@ -4293,7 +4293,7 @@
         <v>970</v>
       </c>
       <c r="B37" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.45">
@@ -4301,7 +4301,7 @@
         <v>971</v>
       </c>
       <c r="B38" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.45">
@@ -4309,7 +4309,7 @@
         <v>972</v>
       </c>
       <c r="B39" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.45">
@@ -4317,7 +4317,7 @@
         <v>973</v>
       </c>
       <c r="B40" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.45">
@@ -4325,7 +4325,7 @@
         <v>974</v>
       </c>
       <c r="B41" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.45">
@@ -4333,7 +4333,7 @@
         <v>975</v>
       </c>
       <c r="B42" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.45">
@@ -4341,7 +4341,7 @@
         <v>976</v>
       </c>
       <c r="B43" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.45">
@@ -4349,7 +4349,7 @@
         <v>977</v>
       </c>
       <c r="B44" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.45">
@@ -4357,7 +4357,7 @@
         <v>978</v>
       </c>
       <c r="B45" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.45">
@@ -4365,7 +4365,7 @@
         <v>979</v>
       </c>
       <c r="B46" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.45">
@@ -4373,7 +4373,7 @@
         <v>980</v>
       </c>
       <c r="B47" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.45">
@@ -4381,7 +4381,7 @@
         <v>981</v>
       </c>
       <c r="B48" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.45">
@@ -4389,7 +4389,7 @@
         <v>982</v>
       </c>
       <c r="B49" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.45">
@@ -4397,7 +4397,7 @@
         <v>983</v>
       </c>
       <c r="B50" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.45">
@@ -4405,7 +4405,7 @@
         <v>984</v>
       </c>
       <c r="B51" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.45">
@@ -4413,7 +4413,7 @@
         <v>985</v>
       </c>
       <c r="B52" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.45">
@@ -4421,7 +4421,7 @@
         <v>986</v>
       </c>
       <c r="B53" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.45">
@@ -4429,7 +4429,7 @@
         <v>987</v>
       </c>
       <c r="B54" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.45">
@@ -4437,7 +4437,7 @@
         <v>937</v>
       </c>
       <c r="B55" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.45">
@@ -4445,7 +4445,7 @@
         <v>938</v>
       </c>
       <c r="B56" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.45">
@@ -4453,7 +4453,7 @@
         <v>939</v>
       </c>
       <c r="B57" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.45">
@@ -4461,7 +4461,7 @@
         <v>940</v>
       </c>
       <c r="B58" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.45">
@@ -4469,7 +4469,7 @@
         <v>941</v>
       </c>
       <c r="B59" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.45">
@@ -4477,7 +4477,7 @@
         <v>942</v>
       </c>
       <c r="B60" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.45">
@@ -4485,7 +4485,7 @@
         <v>943</v>
       </c>
       <c r="B61" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.45">
@@ -4493,7 +4493,7 @@
         <v>944</v>
       </c>
       <c r="B62" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.45">
@@ -4501,7 +4501,7 @@
         <v>945</v>
       </c>
       <c r="B63" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.45">
@@ -4509,7 +4509,7 @@
         <v>946</v>
       </c>
       <c r="B64" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.45">
@@ -4517,7 +4517,7 @@
         <v>947</v>
       </c>
       <c r="B65" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.45">
@@ -4525,7 +4525,7 @@
         <v>948</v>
       </c>
       <c r="B66" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.45">
@@ -4533,7 +4533,7 @@
         <v>949</v>
       </c>
       <c r="B67" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.45">
@@ -4541,7 +4541,7 @@
         <v>950</v>
       </c>
       <c r="B68" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.45">
@@ -4549,7 +4549,7 @@
         <v>951</v>
       </c>
       <c r="B69" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.45">
@@ -4557,7 +4557,7 @@
         <v>952</v>
       </c>
       <c r="B70" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.45">
@@ -4565,7 +4565,7 @@
         <v>953</v>
       </c>
       <c r="B71" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.45">
@@ -4573,7 +4573,7 @@
         <v>954</v>
       </c>
       <c r="B72" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.45">
@@ -4581,7 +4581,7 @@
         <v>955</v>
       </c>
       <c r="B73" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.45">
@@ -4589,7 +4589,7 @@
         <v>956</v>
       </c>
       <c r="B74" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.45">
@@ -4597,7 +4597,7 @@
         <v>957</v>
       </c>
       <c r="B75" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.45">
@@ -4605,7 +4605,7 @@
         <v>958</v>
       </c>
       <c r="B76" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.45">
@@ -4613,7 +4613,7 @@
         <v>959</v>
       </c>
       <c r="B77" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.45">
@@ -4621,7 +4621,7 @@
         <v>960</v>
       </c>
       <c r="B78" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.45">
@@ -4629,7 +4629,7 @@
         <v>961</v>
       </c>
       <c r="B79" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.45">
@@ -4637,7 +4637,7 @@
         <v>962</v>
       </c>
       <c r="B80" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.45">
@@ -4645,7 +4645,7 @@
         <v>988</v>
       </c>
       <c r="B81" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.45">
@@ -4653,7 +4653,7 @@
         <v>989</v>
       </c>
       <c r="B82" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.45">
@@ -4661,7 +4661,7 @@
         <v>990</v>
       </c>
       <c r="B83" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.45">
@@ -4669,7 +4669,7 @@
         <v>991</v>
       </c>
       <c r="B84" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.45">
@@ -4677,7 +4677,7 @@
         <v>992</v>
       </c>
       <c r="B85" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.45">
@@ -4685,7 +4685,7 @@
         <v>993</v>
       </c>
       <c r="B86" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.45">
@@ -4693,7 +4693,7 @@
         <v>994</v>
       </c>
       <c r="B87" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.45">
@@ -4701,7 +4701,7 @@
         <v>995</v>
       </c>
       <c r="B88" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.45">
@@ -4709,7 +4709,7 @@
         <v>996</v>
       </c>
       <c r="B89" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.45">
@@ -4717,7 +4717,7 @@
         <v>997</v>
       </c>
       <c r="B90" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.45">
@@ -4725,7 +4725,7 @@
         <v>998</v>
       </c>
       <c r="B91" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.45">
@@ -4733,7 +4733,7 @@
         <v>999</v>
       </c>
       <c r="B92" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.45">
@@ -4741,7 +4741,7 @@
         <v>1000</v>
       </c>
       <c r="B93" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.45">
@@ -4749,7 +4749,7 @@
         <v>1001</v>
       </c>
       <c r="B94" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.45">
@@ -4757,7 +4757,7 @@
         <v>1002</v>
       </c>
       <c r="B95" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.45">
@@ -4765,7 +4765,7 @@
         <v>1003</v>
       </c>
       <c r="B96" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.45">
@@ -4773,7 +4773,7 @@
         <v>1004</v>
       </c>
       <c r="B97" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.45">
@@ -4781,7 +4781,7 @@
         <v>1005</v>
       </c>
       <c r="B98" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.45">
@@ -4789,7 +4789,7 @@
         <v>1006</v>
       </c>
       <c r="B99" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.45">
@@ -4797,7 +4797,7 @@
         <v>140</v>
       </c>
       <c r="B100" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.45">
@@ -4805,7 +4805,7 @@
         <v>927</v>
       </c>
       <c r="B101" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.45">
@@ -4813,7 +4813,7 @@
         <v>928</v>
       </c>
       <c r="B102" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.45">
@@ -4821,7 +4821,7 @@
         <v>929</v>
       </c>
       <c r="B103" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.45">
@@ -4829,7 +4829,7 @@
         <v>930</v>
       </c>
       <c r="B104" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.45">
@@ -4837,7 +4837,7 @@
         <v>931</v>
       </c>
       <c r="B105" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.45">
@@ -4845,7 +4845,7 @@
         <v>1023</v>
       </c>
       <c r="B106" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.45">
@@ -4853,7 +4853,7 @@
         <v>1024</v>
       </c>
       <c r="B107" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.45">
@@ -4861,7 +4861,7 @@
         <v>1025</v>
       </c>
       <c r="B108" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.45">
@@ -4869,7 +4869,7 @@
         <v>1026</v>
       </c>
       <c r="B109" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.45">
@@ -4877,7 +4877,7 @@
         <v>1027</v>
       </c>
       <c r="B110" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.45">
@@ -4885,7 +4885,7 @@
         <v>1028</v>
       </c>
       <c r="B111" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.45">
@@ -4893,7 +4893,7 @@
         <v>1029</v>
       </c>
       <c r="B112" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.45">
@@ -4901,7 +4901,7 @@
         <v>1030</v>
       </c>
       <c r="B113" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.45">
@@ -4909,7 +4909,7 @@
         <v>1031</v>
       </c>
       <c r="B114" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.45">
@@ -4917,7 +4917,7 @@
         <v>1032</v>
       </c>
       <c r="B115" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.45">
@@ -4925,7 +4925,7 @@
         <v>1033</v>
       </c>
       <c r="B116" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.45">
@@ -4933,7 +4933,7 @@
         <v>1034</v>
       </c>
       <c r="B117" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.45">
@@ -4941,7 +4941,7 @@
         <v>1035</v>
       </c>
       <c r="B118" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.45">
@@ -4949,7 +4949,7 @@
         <v>1036</v>
       </c>
       <c r="B119" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.45">
@@ -4957,7 +4957,7 @@
         <v>1037</v>
       </c>
       <c r="B120" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.45">
@@ -4965,7 +4965,7 @@
         <v>1038</v>
       </c>
       <c r="B121" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.45">
@@ -4973,7 +4973,7 @@
         <v>1039</v>
       </c>
       <c r="B122" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.45">
@@ -4981,7 +4981,7 @@
         <v>1040</v>
       </c>
       <c r="B123" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.45">
@@ -4989,7 +4989,7 @@
         <v>1041</v>
       </c>
       <c r="B124" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.45">
@@ -4997,7 +4997,7 @@
         <v>1042</v>
       </c>
       <c r="B125" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.45">
@@ -5005,7 +5005,7 @@
         <v>1043</v>
       </c>
       <c r="B126" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.45">
@@ -5013,7 +5013,7 @@
         <v>1044</v>
       </c>
       <c r="B127" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.45">
@@ -5021,7 +5021,7 @@
         <v>8</v>
       </c>
       <c r="B128" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prepping for Brute Force Opt
</commit_message>
<xml_diff>
--- a/FlowTracker.xlsx
+++ b/FlowTracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\PHSAhome2.phsabc.ehcnet.ca\Cassidy.Northway\Remote Git\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F747B25-5EFF-4E6C-AC10-EB10999844A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F222552E-8A28-4ECE-AD8C-BF9319FA0DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-4770" windowWidth="18240" windowHeight="28440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3189,27 +3189,12 @@
     <t>0;126;126;0;0.955;0</t>
   </si>
   <si>
-    <t>3;11;11;0;37.90;0</t>
-  </si>
-  <si>
-    <t>4;11;11;0;29.35;0</t>
-  </si>
-  <si>
-    <t>5;11;11;0;68.23;0</t>
-  </si>
-  <si>
     <t>6;63;63;0;5.15;0</t>
   </si>
   <si>
-    <t>7;11;11;0;42.14;0</t>
-  </si>
-  <si>
     <t>29;31;32;0;0;C</t>
   </si>
   <si>
-    <t>8;11;11;0;46.22;0</t>
-  </si>
-  <si>
     <t>9;61;61;0;5.15;0</t>
   </si>
   <si>
@@ -3562,6 +3547,21 @@
   </si>
   <si>
     <t>105;5;5;0;0;0</t>
+  </si>
+  <si>
+    <t>3;11;11;0;18.59;0</t>
+  </si>
+  <si>
+    <t>4;11;11;0;29.36;0</t>
+  </si>
+  <si>
+    <t>5;11;11;0;48.92;0</t>
+  </si>
+  <si>
+    <t>7;11;11;0;22.83;0</t>
+  </si>
+  <si>
+    <t>8;11;11;0;26.91;0</t>
   </si>
 </sst>
 </file>
@@ -4021,7 +4021,7 @@
         <v>935</v>
       </c>
       <c r="B3" t="s">
-        <v>1170</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -4029,7 +4029,7 @@
         <v>817</v>
       </c>
       <c r="B4" t="s">
-        <v>1164</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -4037,7 +4037,7 @@
         <v>844</v>
       </c>
       <c r="B5" t="s">
-        <v>1048</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -4045,7 +4045,7 @@
         <v>845</v>
       </c>
       <c r="B6" t="s">
-        <v>1049</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -4053,7 +4053,7 @@
         <v>818</v>
       </c>
       <c r="B7" t="s">
-        <v>1050</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -4061,7 +4061,7 @@
         <v>807</v>
       </c>
       <c r="B8" t="s">
-        <v>1051</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -4069,7 +4069,7 @@
         <v>819</v>
       </c>
       <c r="B9" t="s">
-        <v>1052</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -4077,7 +4077,7 @@
         <v>846</v>
       </c>
       <c r="B10" t="s">
-        <v>1054</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -4085,7 +4085,7 @@
         <v>811</v>
       </c>
       <c r="B11" t="s">
-        <v>1055</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -4093,7 +4093,7 @@
         <v>848</v>
       </c>
       <c r="B12" t="s">
-        <v>1165</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -4101,7 +4101,7 @@
         <v>847</v>
       </c>
       <c r="B13" t="s">
-        <v>1166</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -4109,7 +4109,7 @@
         <v>1007</v>
       </c>
       <c r="B14" t="s">
-        <v>1056</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -4117,7 +4117,7 @@
         <v>1008</v>
       </c>
       <c r="B15" t="s">
-        <v>1057</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -4125,7 +4125,7 @@
         <v>1009</v>
       </c>
       <c r="B16" t="s">
-        <v>1058</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -4133,7 +4133,7 @@
         <v>1010</v>
       </c>
       <c r="B17" t="s">
-        <v>1059</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -4141,7 +4141,7 @@
         <v>1022</v>
       </c>
       <c r="B18" t="s">
-        <v>1060</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>1011</v>
       </c>
       <c r="B19" t="s">
-        <v>1061</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -4157,7 +4157,7 @@
         <v>1014</v>
       </c>
       <c r="B20" t="s">
-        <v>1062</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -4165,7 +4165,7 @@
         <v>1015</v>
       </c>
       <c r="B21" t="s">
-        <v>1063</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -4173,7 +4173,7 @@
         <v>1016</v>
       </c>
       <c r="B22" t="s">
-        <v>1064</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -4181,7 +4181,7 @@
         <v>1017</v>
       </c>
       <c r="B23" t="s">
-        <v>1065</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -4189,7 +4189,7 @@
         <v>1018</v>
       </c>
       <c r="B24" t="s">
-        <v>1066</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -4197,7 +4197,7 @@
         <v>1019</v>
       </c>
       <c r="B25" t="s">
-        <v>1067</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -4205,7 +4205,7 @@
         <v>1020</v>
       </c>
       <c r="B26" t="s">
-        <v>1068</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -4213,7 +4213,7 @@
         <v>1021</v>
       </c>
       <c r="B27" t="s">
-        <v>1070</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -4221,7 +4221,7 @@
         <v>1012</v>
       </c>
       <c r="B28" t="s">
-        <v>1168</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -4229,7 +4229,7 @@
         <v>1013</v>
       </c>
       <c r="B29" t="s">
-        <v>1169</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -4245,7 +4245,7 @@
         <v>964</v>
       </c>
       <c r="B31" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -4253,7 +4253,7 @@
         <v>965</v>
       </c>
       <c r="B32" t="s">
-        <v>1069</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -4261,7 +4261,7 @@
         <v>966</v>
       </c>
       <c r="B33" t="s">
-        <v>1071</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -4269,7 +4269,7 @@
         <v>967</v>
       </c>
       <c r="B34" t="s">
-        <v>1072</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -4277,7 +4277,7 @@
         <v>968</v>
       </c>
       <c r="B35" t="s">
-        <v>1073</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -4285,7 +4285,7 @@
         <v>969</v>
       </c>
       <c r="B36" t="s">
-        <v>1074</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -4293,7 +4293,7 @@
         <v>970</v>
       </c>
       <c r="B37" t="s">
-        <v>1075</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -4301,7 +4301,7 @@
         <v>971</v>
       </c>
       <c r="B38" t="s">
-        <v>1076</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -4309,7 +4309,7 @@
         <v>972</v>
       </c>
       <c r="B39" t="s">
-        <v>1077</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -4317,7 +4317,7 @@
         <v>973</v>
       </c>
       <c r="B40" t="s">
-        <v>1078</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -4325,7 +4325,7 @@
         <v>974</v>
       </c>
       <c r="B41" t="s">
-        <v>1079</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -4333,7 +4333,7 @@
         <v>975</v>
       </c>
       <c r="B42" t="s">
-        <v>1080</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -4341,7 +4341,7 @@
         <v>976</v>
       </c>
       <c r="B43" t="s">
-        <v>1081</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -4349,7 +4349,7 @@
         <v>977</v>
       </c>
       <c r="B44" t="s">
-        <v>1082</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -4357,7 +4357,7 @@
         <v>978</v>
       </c>
       <c r="B45" t="s">
-        <v>1083</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -4365,7 +4365,7 @@
         <v>979</v>
       </c>
       <c r="B46" t="s">
-        <v>1084</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -4373,7 +4373,7 @@
         <v>980</v>
       </c>
       <c r="B47" t="s">
-        <v>1085</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>981</v>
       </c>
       <c r="B48" t="s">
-        <v>1086</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -4389,7 +4389,7 @@
         <v>982</v>
       </c>
       <c r="B49" t="s">
-        <v>1087</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -4397,7 +4397,7 @@
         <v>983</v>
       </c>
       <c r="B50" t="s">
-        <v>1171</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -4405,7 +4405,7 @@
         <v>984</v>
       </c>
       <c r="B51" t="s">
-        <v>1088</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -4413,7 +4413,7 @@
         <v>985</v>
       </c>
       <c r="B52" t="s">
-        <v>1089</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
@@ -4421,7 +4421,7 @@
         <v>986</v>
       </c>
       <c r="B53" t="s">
-        <v>1090</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
@@ -4429,7 +4429,7 @@
         <v>987</v>
       </c>
       <c r="B54" t="s">
-        <v>1091</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
@@ -4437,7 +4437,7 @@
         <v>937</v>
       </c>
       <c r="B55" t="s">
-        <v>1092</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
@@ -4445,7 +4445,7 @@
         <v>938</v>
       </c>
       <c r="B56" t="s">
-        <v>1093</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
@@ -4453,7 +4453,7 @@
         <v>939</v>
       </c>
       <c r="B57" t="s">
-        <v>1094</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
@@ -4461,7 +4461,7 @@
         <v>940</v>
       </c>
       <c r="B58" t="s">
-        <v>1095</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -4469,7 +4469,7 @@
         <v>941</v>
       </c>
       <c r="B59" t="s">
-        <v>1096</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
@@ -4477,7 +4477,7 @@
         <v>942</v>
       </c>
       <c r="B60" t="s">
-        <v>1097</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -4485,7 +4485,7 @@
         <v>943</v>
       </c>
       <c r="B61" t="s">
-        <v>1098</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -4493,7 +4493,7 @@
         <v>944</v>
       </c>
       <c r="B62" t="s">
-        <v>1099</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -4501,7 +4501,7 @@
         <v>945</v>
       </c>
       <c r="B63" t="s">
-        <v>1100</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -4509,7 +4509,7 @@
         <v>946</v>
       </c>
       <c r="B64" t="s">
-        <v>1101</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -4517,7 +4517,7 @@
         <v>947</v>
       </c>
       <c r="B65" t="s">
-        <v>1102</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -4525,7 +4525,7 @@
         <v>948</v>
       </c>
       <c r="B66" t="s">
-        <v>1103</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
@@ -4533,7 +4533,7 @@
         <v>949</v>
       </c>
       <c r="B67" t="s">
-        <v>1104</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -4541,7 +4541,7 @@
         <v>950</v>
       </c>
       <c r="B68" t="s">
-        <v>1105</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -4549,7 +4549,7 @@
         <v>951</v>
       </c>
       <c r="B69" t="s">
-        <v>1106</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -4557,7 +4557,7 @@
         <v>952</v>
       </c>
       <c r="B70" t="s">
-        <v>1107</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -4565,7 +4565,7 @@
         <v>953</v>
       </c>
       <c r="B71" t="s">
-        <v>1108</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -4573,7 +4573,7 @@
         <v>954</v>
       </c>
       <c r="B72" t="s">
-        <v>1109</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
@@ -4581,7 +4581,7 @@
         <v>955</v>
       </c>
       <c r="B73" t="s">
-        <v>1110</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
@@ -4589,7 +4589,7 @@
         <v>956</v>
       </c>
       <c r="B74" t="s">
-        <v>1111</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
@@ -4597,7 +4597,7 @@
         <v>957</v>
       </c>
       <c r="B75" t="s">
-        <v>1112</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
@@ -4605,7 +4605,7 @@
         <v>958</v>
       </c>
       <c r="B76" t="s">
-        <v>1113</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
@@ -4613,7 +4613,7 @@
         <v>959</v>
       </c>
       <c r="B77" t="s">
-        <v>1114</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
@@ -4621,7 +4621,7 @@
         <v>960</v>
       </c>
       <c r="B78" t="s">
-        <v>1115</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
@@ -4629,7 +4629,7 @@
         <v>961</v>
       </c>
       <c r="B79" t="s">
-        <v>1116</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
@@ -4637,7 +4637,7 @@
         <v>962</v>
       </c>
       <c r="B80" t="s">
-        <v>1117</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
@@ -4645,7 +4645,7 @@
         <v>988</v>
       </c>
       <c r="B81" t="s">
-        <v>1118</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
@@ -4653,7 +4653,7 @@
         <v>989</v>
       </c>
       <c r="B82" t="s">
-        <v>1119</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
@@ -4661,7 +4661,7 @@
         <v>990</v>
       </c>
       <c r="B83" t="s">
-        <v>1120</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
@@ -4669,7 +4669,7 @@
         <v>991</v>
       </c>
       <c r="B84" t="s">
-        <v>1121</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
@@ -4677,7 +4677,7 @@
         <v>992</v>
       </c>
       <c r="B85" t="s">
-        <v>1122</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
@@ -4685,7 +4685,7 @@
         <v>993</v>
       </c>
       <c r="B86" t="s">
-        <v>1123</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
@@ -4693,7 +4693,7 @@
         <v>994</v>
       </c>
       <c r="B87" t="s">
-        <v>1124</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
@@ -4701,7 +4701,7 @@
         <v>995</v>
       </c>
       <c r="B88" t="s">
-        <v>1125</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
@@ -4709,7 +4709,7 @@
         <v>996</v>
       </c>
       <c r="B89" t="s">
-        <v>1126</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
@@ -4717,7 +4717,7 @@
         <v>997</v>
       </c>
       <c r="B90" t="s">
-        <v>1127</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
@@ -4725,7 +4725,7 @@
         <v>998</v>
       </c>
       <c r="B91" t="s">
-        <v>1128</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
@@ -4733,7 +4733,7 @@
         <v>999</v>
       </c>
       <c r="B92" t="s">
-        <v>1129</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
@@ -4741,7 +4741,7 @@
         <v>1000</v>
       </c>
       <c r="B93" t="s">
-        <v>1130</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
@@ -4749,7 +4749,7 @@
         <v>1001</v>
       </c>
       <c r="B94" t="s">
-        <v>1131</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
@@ -4757,7 +4757,7 @@
         <v>1002</v>
       </c>
       <c r="B95" t="s">
-        <v>1132</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
@@ -4765,7 +4765,7 @@
         <v>1003</v>
       </c>
       <c r="B96" t="s">
-        <v>1133</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
@@ -4773,7 +4773,7 @@
         <v>1004</v>
       </c>
       <c r="B97" t="s">
-        <v>1134</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
@@ -4781,7 +4781,7 @@
         <v>1005</v>
       </c>
       <c r="B98" t="s">
-        <v>1135</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
@@ -4789,7 +4789,7 @@
         <v>1006</v>
       </c>
       <c r="B99" t="s">
-        <v>1136</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
@@ -4797,7 +4797,7 @@
         <v>140</v>
       </c>
       <c r="B100" t="s">
-        <v>1137</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
@@ -4805,7 +4805,7 @@
         <v>927</v>
       </c>
       <c r="B101" t="s">
-        <v>1138</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
@@ -4813,7 +4813,7 @@
         <v>928</v>
       </c>
       <c r="B102" t="s">
-        <v>1139</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
@@ -4821,7 +4821,7 @@
         <v>929</v>
       </c>
       <c r="B103" t="s">
-        <v>1140</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
@@ -4829,7 +4829,7 @@
         <v>930</v>
       </c>
       <c r="B104" t="s">
-        <v>1141</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
@@ -4837,7 +4837,7 @@
         <v>931</v>
       </c>
       <c r="B105" t="s">
-        <v>1142</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>1023</v>
       </c>
       <c r="B106" t="s">
-        <v>1143</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
@@ -4853,7 +4853,7 @@
         <v>1024</v>
       </c>
       <c r="B107" t="s">
-        <v>1172</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
@@ -4861,7 +4861,7 @@
         <v>1025</v>
       </c>
       <c r="B108" t="s">
-        <v>1144</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
@@ -4869,7 +4869,7 @@
         <v>1026</v>
       </c>
       <c r="B109" t="s">
-        <v>1145</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
@@ -4877,7 +4877,7 @@
         <v>1027</v>
       </c>
       <c r="B110" t="s">
-        <v>1146</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
@@ -4885,7 +4885,7 @@
         <v>1028</v>
       </c>
       <c r="B111" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
@@ -4893,7 +4893,7 @@
         <v>1029</v>
       </c>
       <c r="B112" t="s">
-        <v>1148</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
@@ -4901,7 +4901,7 @@
         <v>1030</v>
       </c>
       <c r="B113" t="s">
-        <v>1149</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
@@ -4909,7 +4909,7 @@
         <v>1031</v>
       </c>
       <c r="B114" t="s">
-        <v>1150</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
@@ -4917,7 +4917,7 @@
         <v>1032</v>
       </c>
       <c r="B115" t="s">
-        <v>1151</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
@@ -4925,7 +4925,7 @@
         <v>1033</v>
       </c>
       <c r="B116" t="s">
-        <v>1152</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
@@ -4933,7 +4933,7 @@
         <v>1034</v>
       </c>
       <c r="B117" t="s">
-        <v>1153</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
@@ -4941,7 +4941,7 @@
         <v>1035</v>
       </c>
       <c r="B118" t="s">
-        <v>1154</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
@@ -4949,7 +4949,7 @@
         <v>1036</v>
       </c>
       <c r="B119" t="s">
-        <v>1155</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
@@ -4957,7 +4957,7 @@
         <v>1037</v>
       </c>
       <c r="B120" t="s">
-        <v>1156</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
@@ -4965,7 +4965,7 @@
         <v>1038</v>
       </c>
       <c r="B121" t="s">
-        <v>1157</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
@@ -4973,7 +4973,7 @@
         <v>1039</v>
       </c>
       <c r="B122" t="s">
-        <v>1158</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
@@ -4981,7 +4981,7 @@
         <v>1040</v>
       </c>
       <c r="B123" t="s">
-        <v>1159</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
@@ -4989,7 +4989,7 @@
         <v>1041</v>
       </c>
       <c r="B124" t="s">
-        <v>1160</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
@@ -4997,7 +4997,7 @@
         <v>1042</v>
       </c>
       <c r="B125" t="s">
-        <v>1161</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
@@ -5005,7 +5005,7 @@
         <v>1043</v>
       </c>
       <c r="B126" t="s">
-        <v>1162</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
@@ -5013,7 +5013,7 @@
         <v>1044</v>
       </c>
       <c r="B127" t="s">
-        <v>1163</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
@@ -5021,7 +5021,7 @@
         <v>8</v>
       </c>
       <c r="B128" t="s">
-        <v>1167</v>
+        <v>1162</v>
       </c>
     </row>
   </sheetData>
@@ -8980,8 +8980,8 @@
         <v>0.30984615384615383</v>
       </c>
       <c r="E3" s="5">
-        <f>D3*60 +E11</f>
-        <v>37.902510121457489</v>
+        <f>D3*60</f>
+        <v>18.590769230769229</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
@@ -8997,7 +8997,7 @@
         <v>1</v>
       </c>
       <c r="D4">
-        <f t="shared" si="0"/>
+        <f>($H$2*B4)/($I$2*C4)</f>
         <v>0.48923076923076925</v>
       </c>
       <c r="E4" s="5">
@@ -9028,8 +9028,8 @@
         <v>0.81538461538461537</v>
       </c>
       <c r="E5" s="5">
-        <f>D5*60 +E11</f>
-        <v>68.234817813765176</v>
+        <f>D5*60</f>
+        <v>48.92307692307692</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -9087,8 +9087,8 @@
         <v>0.38051282051282048</v>
       </c>
       <c r="E7" s="5">
-        <f>D7*60+E11</f>
-        <v>42.142510121457491</v>
+        <f>D7*60</f>
+        <v>22.830769230769228</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
@@ -9114,8 +9114,8 @@
         <v>0.44846153846153852</v>
       </c>
       <c r="E8" s="5">
-        <f>D8*60 + E11</f>
-        <v>46.219433198380571</v>
+        <f>D8*60</f>
+        <v>26.907692307692312</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
@@ -9424,8 +9424,7 @@
         <v>7.3384615384615381E-2</v>
       </c>
       <c r="E20" s="5">
-        <f t="shared" ref="E20" si="9">D20*60</f>
-        <v>4.4030769230769229</v>
+        <v>0.95499999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fitted Segement work and Organ Contouring
</commit_message>
<xml_diff>
--- a/FlowTracker.xlsx
+++ b/FlowTracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\PHSAhome2.phsabc.ehcnet.ca\Cassidy.Northway\Remote Git\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824E204E-ACC2-438D-ACC6-7EB018D5B9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E329C6BD-785D-4677-A0F1-CE3FF737FB62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-4770" windowWidth="18240" windowHeight="28320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterSheet" sheetId="9" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2898" uniqueCount="1177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2898" uniqueCount="1179">
   <si>
     <t>Filename</t>
   </si>
@@ -3575,6 +3575,12 @@
   </si>
   <si>
     <t>left_gastric_artery, common_hepatic_artery</t>
+  </si>
+  <si>
+    <t>arteries_lleg6, arteries_lleg17</t>
+  </si>
+  <si>
+    <t>arteries_rleg1, arteries_rleg23</t>
   </si>
 </sst>
 </file>
@@ -5359,7 +5365,7 @@
         <v>67</v>
       </c>
       <c r="D18" t="s">
-        <v>106</v>
+        <v>1177</v>
       </c>
       <c r="G18" t="s">
         <v>11</v>
@@ -5466,7 +5472,7 @@
         <v>69</v>
       </c>
       <c r="D25" t="s">
-        <v>679</v>
+        <v>1178</v>
       </c>
       <c r="G25" t="s">
         <v>11</v>

</xml_diff>